<commit_message>
The basic data organization is completed (organizing data under protocols HTTP/1.1, HTTP/2, HTTP/3) and creating result_stummery.xlsx, organizing the mean and sample standard deviation of each data type (for future statistics, drawing line charts and bars, and preparing for the completion of the paper) -Yunlong Wang, Undergraduate , Griffith College Dublin- 2026/7/11 16:47
</commit_message>
<xml_diff>
--- a/results/result_summary.xlsx
+++ b/results/result_summary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wj863\WebstormProjects\Network-Performance-Research\literature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wj863\WebstormProjects\Network-Performance-Research\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1869CA03-8A67-4E72-B823-A57FAFA6A2AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F817927F-C156-47D7-AC89-3F0A037F91EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{426F2216-F02D-450C-8EE8-43E6A120037C}"/>
   </bookViews>
@@ -34,9 +34,138 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+  <si>
+    <t>Average Load Time</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Minimum Load Time</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HTTP/1.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>9.596 s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.55s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>8.06s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HTTP/2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7.346 s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.43s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4.95s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HTTP/3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3.13 s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3.42s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.74s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.19s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.815s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.21s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Standard Deviation(Load Time)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Average TTFB</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>240.56ms</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>230.21ms</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Protocol</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>219.86ms</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Maximum Load Time</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Standard Deviation(TTFB)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>65.02ms</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>85.95ms</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Improvement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>23.5% faster</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>67.4% faster</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Baseline</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,13 +181,69 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="5" tint="-0.249977111117893"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="4" tint="-0.249977111117893"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7C80"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -75,16 +260,115 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="等线"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF7C80"/>
+      <color rgb="FFCC0066"/>
+      <color rgb="FFFF5050"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -94,6 +378,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BEF73E33-0689-4FCB-8B5C-85B4465A0BC5}" name="表3" displayName="表3" ref="A1:H4" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A1:H4" xr:uid="{BEF73E33-0689-4FCB-8B5C-85B4465A0BC5}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{53156296-3DA8-4941-989E-C6104CD9689B}" name="Protocol" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{C76F4AFE-0865-48FF-BB16-AE62632A27B0}" name="Average Load Time" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{617E004E-8DD9-4B17-A878-EC13A2123524}" name="Maximum Load Time" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{4C479B1F-CD5C-4E8F-ADD7-3FEAAA37CA28}" name="Minimum Load Time" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{03CDE097-4CC0-4BB4-B2B5-E97C0E5107FC}" name="Standard Deviation(Load Time)" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{D8A14C0D-87F7-48B1-ABEA-A27B42A40C5F}" name="Average TTFB" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{BCB1E775-273F-4554-AC16-4BE615FA7854}" name="Standard Deviation(TTFB)" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{DD8EECE2-4F63-4B4E-981B-F38B88B8382D}" name="Improvement" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -393,10 +694,128 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A678D222-393D-4675-8A18-02B3B58B557E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.5546875" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="35.33203125" customWidth="1"/>
+    <col min="6" max="6" width="18.88671875" customWidth="1"/>
+    <col min="7" max="7" width="32.88671875" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>